<commit_message>
finish the pipeline for both 9 and 18 month
</commit_message>
<xml_diff>
--- a/RSA analysis/excluded_subs_chair.xlsx
+++ b/RSA analysis/excluded_subs_chair.xlsx
@@ -544,7 +544,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -556,7 +556,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>45</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -592,7 +592,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>79</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -616,7 +616,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>84</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -702,7 +702,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -714,7 +714,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -726,7 +726,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -738,7 +738,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>62</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -774,7 +774,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>80</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -786,7 +786,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>81</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -798,7 +798,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -810,7 +810,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>76</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>36</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -944,7 +944,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -956,7 +956,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>85</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -968,7 +968,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -980,7 +980,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -992,7 +992,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1004,7 +1004,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1016,7 +1016,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>79</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1028,7 +1028,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1040,7 +1040,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1052,7 +1052,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>84</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1186,7 +1186,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1210,7 +1210,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1222,7 +1222,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1234,7 +1234,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>53</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1246,7 +1246,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>81</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1258,7 +1258,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1270,7 +1270,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>76</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1404,7 +1404,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1416,7 +1416,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>36</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1428,7 +1428,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>08</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1452,7 +1452,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1464,7 +1464,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1476,7 +1476,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1488,7 +1488,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1500,7 +1500,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>79</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1512,7 +1512,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1536,7 +1536,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>84</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1694,7 +1694,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1706,7 +1706,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1718,7 +1718,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>62</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1754,7 +1754,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>81</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1766,7 +1766,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1778,7 +1778,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>76</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">

</xml_diff>

<commit_message>
created a new RSA pickle with the undetreded data
</commit_message>
<xml_diff>
--- a/RSA analysis/excluded_subs_chair.xlsx
+++ b/RSA analysis/excluded_subs_chair.xlsx
@@ -520,7 +520,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -544,7 +544,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -556,7 +556,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -568,7 +568,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>08</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -580,7 +580,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>79</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -604,7 +604,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>45</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -616,7 +616,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -702,7 +702,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>80</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -714,7 +714,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -726,7 +726,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -738,7 +738,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>76</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -750,7 +750,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -762,7 +762,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -774,7 +774,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>62</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -786,7 +786,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>81</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -798,7 +798,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>82</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -822,7 +822,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -944,7 +944,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -956,7 +956,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>84</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -968,7 +968,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -980,7 +980,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -992,7 +992,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>36</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1004,7 +1004,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1016,7 +1016,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>08</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1028,7 +1028,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>79</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1040,7 +1040,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1052,7 +1052,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1186,7 +1186,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>53</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1210,7 +1210,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1222,7 +1222,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1234,7 +1234,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>76</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1246,7 +1246,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>81</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1258,7 +1258,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>82</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1270,7 +1270,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1282,7 +1282,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1404,7 +1404,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1416,7 +1416,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1440,7 +1440,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1452,7 +1452,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>36</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1464,7 +1464,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1476,7 +1476,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1488,7 +1488,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>08</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1500,7 +1500,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>79</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1512,7 +1512,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1524,7 +1524,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1536,7 +1536,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1694,7 +1694,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1706,7 +1706,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1718,7 +1718,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1730,7 +1730,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>62</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1742,7 +1742,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>81</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1754,7 +1754,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>76</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1766,7 +1766,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>82</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1778,7 +1778,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1790,7 +1790,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">

</xml_diff>